<commit_message>
Refactor wxPython imports and event handling for no-GUI compatibility; add requirements for Docker; update README for Docker usage
</commit_message>
<xml_diff>
--- a/download/earth_quake_info.xlsx
+++ b/download/earth_quake_info.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,214 +451,214 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2025-05-30 07:17:24</t>
+          <t>2025-05-28 21:34:11</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>44.10</t>
+          <t>13.00</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>87.04</t>
+          <t>145.15</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>新疆昌吉州昌吉市</t>
+          <t>马里亚纳群岛以南海域</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>5.9</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2025-05-30 02:21:34</t>
+          <t>2025-05-28 16:57:48</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>23.72</t>
+          <t>-14.20</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>114.68</t>
+          <t>167.30</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>广东河源市源城区</t>
+          <t>瓦努阿图群岛</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2025-05-29 13:17:07</t>
+          <t>2025-05-28 13:48:12</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>23.71</t>
+          <t>41.26</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>114.69</t>
+          <t>83.73</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>17</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>广东河源市源城区</t>
+          <t>新疆阿克苏地区库车市</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2025-05-28 21:34:11</t>
+          <t>2025-05-28 09:12:57</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>13.00</t>
+          <t>29.30</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>145.15</t>
+          <t>98.78</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>马里亚纳群岛以南海域</t>
+          <t>西藏昌都市芒康县</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>5.9</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2025-05-28 16:57:48</t>
+          <t>2025-05-28 07:21:23</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>-14.20</t>
+          <t>24.16</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>167.30</t>
+          <t>99.41</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>瓦努阿图群岛</t>
+          <t>云南临沧市永德县</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2025-05-28 13:48:12</t>
+          <t>2025-05-28 00:46:02</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>41.26</t>
+          <t>34.65</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>83.73</t>
+          <t>80.70</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>新疆阿克苏地区库车市</t>
+          <t>西藏阿里地区日土县</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2025-05-28 09:12:57</t>
+          <t>2025-05-27 23:27:10</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>29.30</t>
+          <t>34.58</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>98.78</t>
+          <t>80.66</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -668,29 +668,29 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>西藏昌都市芒康县</t>
+          <t>西藏阿里地区日土县</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2025-05-28 07:21:23</t>
+          <t>2025-05-27 11:40:06</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>24.16</t>
+          <t>42.23</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>99.41</t>
+          <t>80.62</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -700,61 +700,61 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>云南临沧市永德县</t>
+          <t>新疆阿克苏地区温宿县</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>5.7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2025-05-28 00:46:02</t>
+          <t>2025-05-26 11:50:20</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>34.65</t>
+          <t>-19.60</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>80.70</t>
+          <t>-69.60</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>100</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>西藏阿里地区日土县</t>
+          <t>智利北部</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2025-05-27 23:27:10</t>
+          <t>2025-05-25 18:49:51</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>34.58</t>
+          <t>-22.75</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>80.66</t>
+          <t>-175.60</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -764,29 +764,29 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>西藏阿里地区日土县</t>
+          <t>斐济群岛以南海域</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2025-05-27 11:40:06</t>
+          <t>2025-05-24 00:33:23</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>42.23</t>
+          <t>-56.60</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>80.62</t>
+          <t>147.55</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -796,285 +796,285 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>新疆阿克苏地区温宿县</t>
+          <t>麦夸里岛以西海域</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>5.7</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2025-05-26 11:50:20</t>
+          <t>2025-05-23 11:57:21</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>-19.60</t>
+          <t>29.03</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>-69.60</t>
+          <t>87.03</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>智利北部</t>
+          <t>西藏日喀则市定日县</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>5.8</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2025-05-25 18:49:51</t>
+          <t>2025-05-23 03:52:35</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>-22.75</t>
+          <t>-4.45</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>-175.60</t>
+          <t>102.00</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>40</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>斐济群岛以南海域</t>
+          <t>印尼苏门答腊岛西南部海域</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2025-05-24 00:33:23</t>
+          <t>2025-05-22 17:21:03</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>-56.60</t>
+          <t>30.90</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>147.55</t>
+          <t>98.92</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>麦夸里岛以西海域</t>
+          <t>四川甘孜州白玉县</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2025-05-23 11:57:21</t>
+          <t>2025-05-22 11:19:35</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>29.03</t>
+          <t>35.70</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>87.03</t>
+          <t>25.80</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>70</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>西藏日喀则市定日县</t>
+          <t>爱琴海</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>5.8</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2025-05-23 03:52:35</t>
+          <t>2025-05-22 07:16:51</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>-4.45</t>
+          <t>34.42</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>102.00</t>
+          <t>104.80</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>印尼苏门答腊岛西南部海域</t>
+          <t>甘肃定西市岷县</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>3.7</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2025-05-22 17:21:03</t>
+          <t>2025-05-22 00:50:20</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>30.90</t>
+          <t>28.34</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>98.92</t>
+          <t>104.55</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>四川甘孜州白玉县</t>
+          <t>四川宜宾市高县</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2025-05-22 11:19:35</t>
+          <t>2025-05-21 02:53:39</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>35.70</t>
+          <t>32.01</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>25.80</t>
+          <t>97.32</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>爱琴海</t>
+          <t>西藏昌都市卡若区</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2025-05-22 07:16:51</t>
+          <t>2025-05-21 00:29:52</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>34.42</t>
+          <t>27.14</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>104.80</t>
+          <t>102.96</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>17</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>甘肃定西市岷县</t>
+          <t>云南昭通市巧家县</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3.7</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2025-05-22 00:50:20</t>
+          <t>2025-05-20 23:06:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>28.34</t>
+          <t>-3.80</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>104.55</t>
+          <t>144.85</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1084,29 +1084,29 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>四川宜宾市高县</t>
+          <t>巴布亚新几内亚附近海域</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2025-05-21 02:53:39</t>
+          <t>2025-05-20 02:03:14</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>32.01</t>
+          <t>41.74</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>97.32</t>
+          <t>88.22</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1116,61 +1116,61 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>西藏昌都市卡若区</t>
+          <t>新疆巴音郭楞州和硕县</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2025-05-21 00:29:52</t>
+          <t>2025-05-20 00:41:12</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>27.14</t>
+          <t>41.28</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>102.96</t>
+          <t>84.01</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>云南昭通市巧家县</t>
+          <t>新疆阿克苏地区库车市</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2025-05-20 23:06:00</t>
+          <t>2025-05-19 20:00:06</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>-3.80</t>
+          <t>28.42</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>144.85</t>
+          <t>87.46</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1180,61 +1180,61 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>巴布亚新几内亚附近海域</t>
+          <t>西藏日喀则市定日县</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2025-05-20 02:03:14</t>
+          <t>2025-05-19 12:58:35</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>41.74</t>
+          <t>32.80</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>88.22</t>
+          <t>101.20</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>新疆巴音郭楞州和硕县</t>
+          <t>青海果洛州班玛县</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2025-05-20 00:41:12</t>
+          <t>2025-05-19 01:30:30</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>41.28</t>
+          <t>33.83</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>84.01</t>
+          <t>90.38</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1244,29 +1244,29 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>新疆阿克苏地区库车市</t>
+          <t>青海海西州唐古拉地区</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2025-05-19 20:00:06</t>
+          <t>2025-05-18 07:36:31</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>28.42</t>
+          <t>28.92</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>87.46</t>
+          <t>95.82</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1276,125 +1276,125 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>西藏日喀则市定日县</t>
+          <t>西藏林芝市墨脱县</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2025-05-19 12:58:35</t>
+          <t>2025-05-17 23:54:49</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>32.80</t>
+          <t>21.30</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>101.20</t>
+          <t>96.05</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>青海果洛州班玛县</t>
+          <t>缅甸</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2025-05-19 01:30:30</t>
+          <t>2025-05-17 18:22:13</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>33.83</t>
+          <t>-14.70</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>90.38</t>
+          <t>-74.30</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>100</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>青海海西州唐古拉地区</t>
+          <t>秘鲁</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2025-05-18 07:36:31</t>
+          <t>2025-05-16 19:37:10</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>28.92</t>
+          <t>39.70</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>95.82</t>
+          <t>82.93</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>西藏林芝市墨脱县</t>
+          <t>新疆阿克苏地区沙雅县</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2025-05-17 23:54:49</t>
+          <t>2025-05-16 19:02:45</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>21.30</t>
+          <t>37.61</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>96.05</t>
+          <t>115.13</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1404,125 +1404,125 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>缅甸</t>
+          <t>河北邢台市宁晋县</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2025-05-17 18:22:13</t>
+          <t>2025-05-16 09:00:07</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>-14.70</t>
+          <t>25.12</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>-74.30</t>
+          <t>98.13</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>秘鲁</t>
+          <t>云南德宏州盈江县</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2025-05-16 19:37:10</t>
+          <t>2025-05-15 22:33:02</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>39.70</t>
+          <t>23.36</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>82.93</t>
+          <t>118.50</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>新疆阿克苏地区沙雅县</t>
+          <t>台湾海峡</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2025-05-16 19:02:45</t>
+          <t>2025-05-14 12:15:37</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>37.61</t>
+          <t>-18.70</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>115.13</t>
+          <t>-175.10</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>240</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>河北邢台市宁晋县</t>
+          <t>汤加群岛</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2025-05-16 09:00:07</t>
+          <t>2025-05-14 12:14:22</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>25.12</t>
+          <t>29.03</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>98.13</t>
+          <t>87.03</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1532,93 +1532,93 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>云南德宏州盈江县</t>
+          <t>西藏日喀则市定日县</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2025-05-15 22:33:02</t>
+          <t>2025-05-14 06:51:14</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>23.36</t>
+          <t>35.20</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>118.50</t>
+          <t>27.10</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>70</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>台湾海峡</t>
+          <t>希腊克里特岛附近海域</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>6.4</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2025-05-14 12:15:37</t>
+          <t>2025-05-13 08:01:55</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>-18.70</t>
+          <t>30.84</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>-175.10</t>
+          <t>98.96</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>汤加群岛</t>
+          <t>四川甘孜州白玉县</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2025-05-14 12:14:22</t>
+          <t>2025-05-12 06:33:18</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>29.03</t>
+          <t>41.40</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>87.03</t>
+          <t>78.88</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1628,71 +1628,71 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>西藏日喀则市定日县</t>
+          <t>新疆阿克苏地区乌什县</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2025-05-14 06:51:14</t>
+          <t>2025-05-12 05:50:01</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>35.20</t>
+          <t>62.80</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>27.10</t>
+          <t>178.55</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>30</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>希腊克里特岛附近海域</t>
+          <t>俄罗斯西伯利亚东部</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2025-05-13 08:01:55</t>
+          <t>2025-05-12 05:11:21</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>30.84</t>
+          <t>28.91</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>98.96</t>
+          <t>87.54</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>四川甘孜州白玉县</t>
+          <t>西藏日喀则市拉孜县</t>
         </is>
       </c>
     </row>
@@ -1704,241 +1704,241 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2025-05-12 06:33:18</t>
+          <t>2025-05-12 00:31:49</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>41.40</t>
+          <t>41.32</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>78.88</t>
+          <t>83.28</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>新疆阿克苏地区乌什县</t>
+          <t>新疆阿克苏地区库车市</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>5.7</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2025-05-12 05:50:01</t>
+          <t>2025-05-11 19:22:22</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>62.80</t>
+          <t>-17.55</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>178.55</t>
+          <t>168.20</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>俄罗斯西伯利亚东部</t>
+          <t>瓦努阿图群岛</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>5.9</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2025-05-12 05:11:21</t>
+          <t>2025-05-11 16:57:42</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>28.91</t>
+          <t>3.70</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>87.54</t>
+          <t>96.95</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>80</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>西藏日喀则市拉孜县</t>
+          <t>印尼苏门答腊岛</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2025-05-12 00:31:49</t>
+          <t>2025-05-11 16:09:14</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>41.32</t>
+          <t>40.90</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>83.28</t>
+          <t>78.08</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>新疆阿克苏地区库车市</t>
+          <t>新疆克孜勒苏州阿合奇县</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>5.7</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2025-05-11 19:22:22</t>
+          <t>2025-05-10 09:33:07</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>-17.55</t>
+          <t>34.11</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>168.20</t>
+          <t>86.47</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>瓦努阿图群岛</t>
+          <t>西藏那曲市尼玛县</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>5.9</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2025-05-11 16:57:42</t>
+          <t>2025-05-10 00:38:53</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>3.70</t>
+          <t>41.19</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>96.95</t>
+          <t>83.72</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>印尼苏门答腊岛</t>
+          <t>新疆阿克苏地区库车市</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2025-05-11 16:09:14</t>
+          <t>2025-05-09 14:25:50</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>40.90</t>
+          <t>41.86</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>78.08</t>
+          <t>89.05</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>新疆克孜勒苏州阿合奇县</t>
+          <t>新疆吐鲁番市托克逊县</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2025-05-10 09:33:07</t>
+          <t>2025-05-09 09:41:56</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>34.11</t>
+          <t>34.46</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>86.47</t>
+          <t>93.19</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -1948,349 +1948,349 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>西藏那曲市尼玛县</t>
+          <t>青海玉树州治多县</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2025-05-10 00:38:53</t>
+          <t>2025-05-09 05:51:50</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>41.19</t>
+          <t>41.80</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>83.72</t>
+          <t>81.69</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>新疆阿克苏地区库车市</t>
+          <t>新疆阿克苏地区拜城县</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2025-05-09 14:25:50</t>
+          <t>2025-05-08 22:48:35</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>41.86</t>
+          <t>29.02</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>89.05</t>
+          <t>87.02</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>新疆吐鲁番市托克逊县</t>
+          <t>西藏日喀则市定日县</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2025-05-09 09:41:56</t>
+          <t>2025-05-07 03:43:29</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>34.46</t>
+          <t>41.13</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>93.19</t>
+          <t>83.75</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>青海玉树州治多县</t>
+          <t>新疆阿克苏地区库车市</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2025-05-09 05:51:50</t>
+          <t>2025-05-06 16:08:26</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>41.80</t>
+          <t>39.32</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>81.69</t>
+          <t>73.43</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>新疆阿克苏地区拜城县</t>
+          <t>塔吉克斯坦</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>5.7</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2025-05-08 22:48:35</t>
+          <t>2025-05-05 18:53:27</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>29.02</t>
+          <t>23.87</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>87.02</t>
+          <t>121.94</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>西藏日喀则市定日县</t>
+          <t>台湾花莲县海域</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2025-05-07 03:43:29</t>
+          <t>2025-05-05 18:10:01</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>41.13</t>
+          <t>23.89</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>83.75</t>
+          <t>121.94</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>16</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>新疆阿克苏地区库车市</t>
+          <t>台湾花莲县海域</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>5.8</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2025-05-06 16:08:26</t>
+          <t>2025-05-05 16:28:14</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>39.32</t>
+          <t>16.50</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>73.43</t>
+          <t>-92.65</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>260</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>塔吉克斯坦</t>
+          <t>墨西哥</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>5.7</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2025-05-05 18:53:27</t>
+          <t>2025-05-04 14:45:43</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>23.87</t>
+          <t>41.91</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>121.94</t>
+          <t>82.35</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>台湾花莲县海域</t>
+          <t>新疆阿克苏地区拜城县</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2025-05-05 18:10:01</t>
+          <t>2025-05-03 21:31:44</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>23.89</t>
+          <t>28.60</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>121.94</t>
+          <t>87.46</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>台湾花莲县海域</t>
+          <t>西藏日喀则市定日县</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>5.8</t>
+          <t>5.7</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2025-05-05 16:28:14</t>
+          <t>2025-05-03 20:51:45</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16.50</t>
+          <t>0.40</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>-92.65</t>
+          <t>121.70</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>120</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>墨西哥</t>
+          <t>印尼托米尼湾</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2025-05-04 14:45:43</t>
+          <t>2025-05-03 15:54:05</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>41.91</t>
+          <t>33.60</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>82.35</t>
+          <t>81.92</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2300,29 +2300,29 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>新疆阿克苏地区拜城县</t>
+          <t>西藏阿里地区日土县</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2025-05-03 21:31:44</t>
+          <t>2025-05-03 01:59:09</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>28.60</t>
+          <t>-57.20</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>87.46</t>
+          <t>-67.10</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2332,199 +2332,263 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>西藏日喀则市定日县</t>
+          <t>德雷克海峡</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>5.7</t>
+          <t>7.4</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2025-05-03 20:51:45</t>
+          <t>2025-05-02 20:58:25</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.40</t>
+          <t>-56.80</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>121.70</t>
+          <t>-68.25</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>印尼托米尼湾</t>
+          <t>德雷克海峡</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2025-05-03 15:54:05</t>
+          <t>2025-05-02 18:59:22</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>33.60</t>
+          <t>-7.30</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>81.92</t>
+          <t>156.15</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>30</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>西藏阿里地区日土县</t>
+          <t>所罗门群岛</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>6.4</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2025-05-03 01:59:09</t>
+          <t>2025-05-02 00:04:55</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>-57.20</t>
+          <t>-28.55</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>-67.10</t>
+          <t>-67.35</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>30</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>德雷克海峡</t>
+          <t>阿根廷</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>7.4</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2025-05-02 20:58:25</t>
+          <t>2025-04-30 00:41:34</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>-56.80</t>
+          <t>41.14</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>-68.25</t>
+          <t>83.75</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>德雷克海峡</t>
+          <t>新疆阿克苏地区库车市</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2025-05-02 18:59:22</t>
+          <t>2025-04-29 22:53:37</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>-7.30</t>
+          <t>-54.20</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>156.15</t>
+          <t>155.40</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>所罗门群岛</t>
+          <t>麦夸里岛附近海域</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2025-05-02 00:04:55</t>
+          <t>2025-04-29 21:16:33</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>-28.55</t>
+          <t>-48.40</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>-67.35</t>
+          <t>165.25</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>阿根廷</t>
+          <t>新西兰南岛西岸远海</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>3.8</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2025-04-29 16:20:32</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>33.62</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>81.92</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>西藏阿里地区日土县</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2025-04-29 16:17:23</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>33.58</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>81.93</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>西藏阿里地区日土县</t>
         </is>
       </c>
     </row>

</xml_diff>